<commit_message>
VCS1: loadTestIncrementPhase gains seating; properties loading_phase carries valueCodeSpace; converter reads an optional ValueCodeSpace column
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Codelist Excel Files and Conversion Templates to XML/loadTestIncrementPhase.xlsx
+++ b/Codelist Excel Files and Conversion Templates to XML/loadTestIncrementPhase.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="9200" yWindow="3280" windowWidth="39400" windowHeight="24940" tabRatio="500" firstSheet="0" activeTab="4" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="DictionaryName" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Definitions" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="AssociatedElements" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="AlternateNames" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Lists" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DictionaryName" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Definitions" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AssociatedElements" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AlternateNames" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -985,7 +985,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Codes classifying whether a load test increment is part of loading, unloading, or a reload within a cyclic sequence. Used for the value of diggs:LoadTestIncrementType/loadingPhase.</t>
+          <t>Codes classifying whether a load test increment is part of seating, loading, unloading, or a reload within a cyclic sequence. Used for the value of diggs:LoadTestIncrementType/loadingPhase.</t>
         </is>
       </c>
     </row>
@@ -995,7 +995,7 @@
       <c r="D4" s="2" t="n"/>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
     </row>
@@ -1170,12 +1170,32 @@
         <f>IF(ISNA(VLOOKUP(B5,AssociatedElements!B$2:B2943,1,FALSE)),"Not used","")</f>
         <v/>
       </c>
-      <c r="B5" s="13" t="n"/>
-      <c r="C5" s="13" t="n"/>
-      <c r="D5" s="14" t="n"/>
-      <c r="E5" s="13" t="n"/>
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>seating</t>
+        </is>
+      </c>
+      <c r="C5" s="13" t="inlineStr">
+        <is>
+          <t>Seating</t>
+        </is>
+      </c>
+      <c r="D5" s="14" t="inlineStr">
+        <is>
+          <t>The increment belongs to the seating or pre-loading cycle applied before the test proper - the seating load being applied or, afterwards, released - and its settlement is not part of the loading curve.</t>
+        </is>
+      </c>
+      <c r="E5" s="13" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
       <c r="F5" s="13" t="n"/>
-      <c r="G5" s="9" t="n"/>
+      <c r="G5" s="9" t="inlineStr">
+        <is>
+          <t>DIGGS</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2">
@@ -1635,7 +1655,16 @@
         <f>IF(ISNA(VLOOKUP(B5,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B5" s="2" t="n"/>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>seating</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>//diggs:LoadTestIncrement/diggs:loadingPhase</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6">

</xml_diff>